<commit_message>
TEST AND MODIFICATIONS FOR NEW INVENTORY SCREEN
</commit_message>
<xml_diff>
--- a/LISTADO_INICIAL_ALTA_MATERIALES_BLANKET.xlsx
+++ b/LISTADO_INICIAL_ALTA_MATERIALES_BLANKET.xlsx
@@ -8,12 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\alejandrod\Documents\GitHub\MATERIALS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{35487082-40DD-44EC-B6A6-053D9340302F}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{62225162-5DBB-43C2-92F6-BD6C7BDB7675}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19092" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{4AC2D1D3-BA54-402C-89E2-8E241129B71B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" tabRatio="220" activeTab="2" xr2:uid="{4AC2D1D3-BA54-402C-89E2-8E241129B71B}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Hoja2" sheetId="2" r:id="rId2"/>
+    <sheet name="20200812" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="211" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="491" uniqueCount="232">
   <si>
     <t>#ITEM</t>
   </si>
@@ -513,13 +515,240 @@
   </si>
   <si>
     <t>4.5543/LY</t>
+  </si>
+  <si>
+    <t>PROVEEDOR</t>
+  </si>
+  <si>
+    <t>DESCRIPCION</t>
+  </si>
+  <si>
+    <t>IDENTIFICACION DE  MATERIALES( MANUEL G)</t>
+  </si>
+  <si>
+    <t>#PART PROVEEDOR</t>
+  </si>
+  <si>
+    <t>#PART PEARL</t>
+  </si>
+  <si>
+    <t>FXI </t>
+  </si>
+  <si>
+    <t>A173-040 EL 10 MM 27KG/M3 (1.7PCF) PUR FOAM + SCRIM +SPUNFAB ADHESIVE</t>
+  </si>
+  <si>
+    <t>A173-040 EL 3MM 27KG/M3 (1.7PCF) PUR FOAM + SCRIM +SPUNFAB ADHESIVE</t>
+  </si>
+  <si>
+    <t>A  200-060</t>
+  </si>
+  <si>
+    <t>A2000-060 EL SPUNFAB PA1541 , 0.9OZ 60”X 6.00 MM , WITH TB16 SCRIM</t>
+  </si>
+  <si>
+    <t>FXWSA262</t>
+  </si>
+  <si>
+    <t>A195-038 EL FOAM SPUNFAB PA1541 0.9OZ. 0.0984" X 60" 2.5MM - UNBACKED</t>
+  </si>
+  <si>
+    <t>FXWSA190</t>
+  </si>
+  <si>
+    <t>A195-038 EL FOAM TB16 (ADHESIVE) SPUNFAB PA1541 0.9OZ. 0.1220" X  60"  3.1 MM</t>
+  </si>
+  <si>
+    <t>FXWSA193</t>
+  </si>
+  <si>
+    <t>3 MESH SPACER FABRIC T6035, 6MM THICKNESS, 59´ ROLL WIDTH - BLACK  WITH SPUNFAB PA 1301 0.7 OSY (WEB)</t>
+  </si>
+  <si>
+    <t>T6035-0600-1500-0109 WEBH</t>
+  </si>
+  <si>
+    <t>3 MESH SPACER FABRIC T6126, 10MM THICKNESS, 59´ ROLL WIDTH - BLACK  WITH SPUNFAB PA 1301 0.7 OSY (WEB)</t>
+  </si>
+  <si>
+    <t>T6126-1000-1570-0109 WEBH</t>
+  </si>
+  <si>
+    <t>D4922-35-270(77003 6230361)</t>
+  </si>
+  <si>
+    <t>HGFSB361</t>
+  </si>
+  <si>
+    <t>D4922-45-250(77006 6250340)</t>
+  </si>
+  <si>
+    <t>HGRSB340</t>
+  </si>
+  <si>
+    <t>D4922-40-270(77009 6240369)</t>
+  </si>
+  <si>
+    <t>HGFSC369</t>
+  </si>
+  <si>
+    <t>D4922-45-265 (77016 6260359 (2)</t>
+  </si>
+  <si>
+    <t>HGRSC359</t>
+  </si>
+  <si>
+    <t>KUFNER BD1103NA71A150 (BLACK)</t>
+  </si>
+  <si>
+    <t>KUFNER R179G46150 (BLACK)</t>
+  </si>
+  <si>
+    <t>KUFNER TK1080B1801095 (BLACK)</t>
+  </si>
+  <si>
+    <t>KUFNER R659G46150 (BLACK)</t>
+  </si>
+  <si>
+    <t>THREAD T90 BLACK TX7/DX9</t>
+  </si>
+  <si>
+    <t>AET90DX9</t>
+  </si>
+  <si>
+    <t>THREAD T90 CARAMEL LK5</t>
+  </si>
+  <si>
+    <t>AET90LK5</t>
+  </si>
+  <si>
+    <t>THREAD T90 TUPELO WT5</t>
+  </si>
+  <si>
+    <t>AET90WT5</t>
+  </si>
+  <si>
+    <t>THREAD T90 COGNAC WU9</t>
+  </si>
+  <si>
+    <t>AET90WUC</t>
+  </si>
+  <si>
+    <t>THREAD T90 BLUE AGAVE WA6</t>
+  </si>
+  <si>
+    <r>
+      <t>AET9</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FFFF0000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+      </rPr>
+      <t>0WA6</t>
+    </r>
+  </si>
+  <si>
+    <t>THREAD T90 SEA SALT SA5</t>
+  </si>
+  <si>
+    <t>AET90SA5</t>
+  </si>
+  <si>
+    <t>RETICULADO</t>
+  </si>
+  <si>
+    <t>FXCF60MM</t>
+  </si>
+  <si>
+    <t>VS63XSD4</t>
+  </si>
+  <si>
+    <t>VS66BWA6</t>
+  </si>
+  <si>
+    <t>VS63BWT5</t>
+  </si>
+  <si>
+    <t>VS66VTX7</t>
+  </si>
+  <si>
+    <t>VCFCATX7</t>
+  </si>
+  <si>
+    <t>VCFCASD4</t>
+  </si>
+  <si>
+    <t>VCFCPRX7</t>
+  </si>
+  <si>
+    <t>#ITEM PEARL</t>
+  </si>
+  <si>
+    <t>FXIRUWL62</t>
+  </si>
+  <si>
+    <t>FXYL10M2 - FCXI173</t>
+  </si>
+  <si>
+    <t>A195-038 EL</t>
+  </si>
+  <si>
+    <t>FXIWPI 2059662 63*3 MM UNBACKED SIN SCRIM</t>
+  </si>
+  <si>
+    <t>SISTEMAS PEARL</t>
+  </si>
+  <si>
+    <t>FXIJLSUM 2013995 3mm 27kg/M3(1.7PCF) PUR FOAM+TB16</t>
+  </si>
+  <si>
+    <t>FXIRUWL 2114786 RUPIN Y WLA173040EL 60*6mm SPUNFAB</t>
+  </si>
+  <si>
+    <t>A2000-060EL SPUNF PA1541 .9OZ 60X6MM, W/TB16 SCRIM</t>
+  </si>
+  <si>
+    <t>A200-060 EL</t>
+  </si>
+  <si>
+    <t>D4922-35-270</t>
+  </si>
+  <si>
+    <t>D4922-45-250</t>
+  </si>
+  <si>
+    <t>D4922-40-270</t>
+  </si>
+  <si>
+    <t>D4922-45-265</t>
+  </si>
+  <si>
+    <t>D4922-35-270 (40X270MM) CLEAR BEAD</t>
+  </si>
+  <si>
+    <t>D4922-40-270 (45X280MM) BLUE BEAD</t>
+  </si>
+  <si>
+    <t>D4922-45-250 (55X250MM) CLEAR BEAD</t>
+  </si>
+  <si>
+    <t>D4922-45-265 (55X265MM) BLUE BEAD</t>
+  </si>
+  <si>
+    <t>lb</t>
+  </si>
+  <si>
+    <t>pcs</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="10" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -586,8 +815,33 @@
       <name val="Calibri"/>
       <family val="2"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FFFF0000"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="9">
+  <fills count="12">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -636,8 +890,26 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF000000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFFFF"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="15">
+  <borders count="16">
     <border>
       <left/>
       <right/>
@@ -815,11 +1087,24 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color rgb="FF000000"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="86">
+  <cellXfs count="138">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -837,24 +1122,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1046,6 +1313,149 @@
     <xf numFmtId="0" fontId="1" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="10" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1055,13 +1465,40 @@
     <xf numFmtId="0" fontId="8" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1382,7 +1819,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="12.7109375" style="5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="63.140625" style="5" customWidth="1"/>
+    <col min="3" max="3" width="66.85546875" style="5" customWidth="1"/>
     <col min="4" max="4" width="62.28515625" customWidth="1"/>
     <col min="5" max="6" width="25.42578125" customWidth="1"/>
     <col min="7" max="7" width="19.42578125" customWidth="1"/>
@@ -1391,321 +1828,321 @@
     <col min="10" max="10" width="23.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:9" s="22" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B1" s="24" t="s">
+    <row r="1" spans="2:9" s="16" customFormat="1" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="18" t="s">
         <v>0</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="D1" s="20" t="s">
-        <v>1</v>
-      </c>
-      <c r="E1" s="20" t="s">
+      <c r="D1" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="E1" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="F1" s="20" t="s">
+      <c r="F1" s="14" t="s">
         <v>112</v>
       </c>
-      <c r="G1" s="21" t="s">
+      <c r="G1" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="H1" s="20" t="s">
+      <c r="H1" s="14" t="s">
         <v>59</v>
       </c>
-      <c r="I1" s="20" t="s">
+      <c r="I1" s="14" t="s">
         <v>60</v>
       </c>
     </row>
     <row r="2" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B2" s="25">
+      <c r="B2" s="19">
         <v>28</v>
       </c>
-      <c r="C2" s="18" t="s">
+      <c r="C2" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="D2" s="28"/>
-      <c r="E2" s="32" t="s">
+      <c r="D2" s="22"/>
+      <c r="E2" s="26" t="s">
         <v>62</v>
       </c>
-      <c r="F2" s="32" t="s">
+      <c r="F2" s="26" t="s">
         <v>41</v>
       </c>
-      <c r="G2" s="33" t="s">
+      <c r="G2" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H2" s="19" t="s">
+      <c r="H2" s="13" t="s">
         <v>64</v>
       </c>
-      <c r="I2" s="32" t="s">
+      <c r="I2" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="3" spans="2:9" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="25">
+      <c r="B3" s="19">
         <v>67</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="C3" s="23" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="28"/>
-      <c r="E3" s="32" t="s">
+      <c r="D3" s="22"/>
+      <c r="E3" s="26" t="s">
         <v>37</v>
       </c>
-      <c r="F3" s="32" t="s">
+      <c r="F3" s="26" t="s">
         <v>38</v>
       </c>
-      <c r="G3" s="33" t="s">
+      <c r="G3" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H3" s="19" t="s">
+      <c r="H3" s="13" t="s">
         <v>67</v>
       </c>
-      <c r="I3" s="32" t="s">
+      <c r="I3" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="4" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B4" s="25">
+      <c r="B4" s="19">
         <v>69</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="12" t="s">
         <v>68</v>
       </c>
-      <c r="D4" s="28"/>
-      <c r="E4" s="32" t="s">
+      <c r="D4" s="22"/>
+      <c r="E4" s="26" t="s">
         <v>69</v>
       </c>
-      <c r="F4" s="32" t="s">
+      <c r="F4" s="26" t="s">
         <v>70</v>
       </c>
-      <c r="G4" s="33" t="s">
+      <c r="G4" s="27" t="s">
         <v>71</v>
       </c>
-      <c r="H4" s="19"/>
-      <c r="I4" s="32" t="s">
+      <c r="H4" s="13"/>
+      <c r="I4" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="5" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B5" s="25">
+      <c r="B5" s="19">
         <v>70</v>
       </c>
-      <c r="C5" s="18" t="s">
+      <c r="C5" s="12" t="s">
         <v>72</v>
       </c>
-      <c r="D5" s="28"/>
-      <c r="E5" s="32"/>
-      <c r="F5" s="32" t="s">
+      <c r="D5" s="22"/>
+      <c r="E5" s="26"/>
+      <c r="F5" s="26" t="s">
         <v>53</v>
       </c>
-      <c r="G5" s="33" t="s">
+      <c r="G5" s="27" t="s">
         <v>73</v>
       </c>
-      <c r="H5" s="19"/>
-      <c r="I5" s="32" t="s">
+      <c r="H5" s="13"/>
+      <c r="I5" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="6" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="25">
+      <c r="B6" s="19">
         <v>82</v>
       </c>
-      <c r="C6" s="18" t="s">
+      <c r="C6" s="12" t="s">
         <v>74</v>
       </c>
-      <c r="D6" s="28"/>
-      <c r="E6" s="32" t="s">
+      <c r="D6" s="22"/>
+      <c r="E6" s="26" t="s">
         <v>34</v>
       </c>
-      <c r="F6" s="32" t="s">
+      <c r="F6" s="26" t="s">
         <v>35</v>
       </c>
-      <c r="G6" s="33" t="s">
+      <c r="G6" s="27" t="s">
         <v>63</v>
       </c>
-      <c r="H6" s="19" t="s">
+      <c r="H6" s="13" t="s">
         <v>75</v>
       </c>
-      <c r="I6" s="32" t="s">
+      <c r="I6" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="7" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="25">
+      <c r="B7" s="19">
         <v>176</v>
       </c>
-      <c r="C7" s="18" t="s">
+      <c r="C7" s="12" t="s">
         <v>76</v>
       </c>
-      <c r="D7" s="28"/>
-      <c r="E7" s="32" t="s">
+      <c r="D7" s="22"/>
+      <c r="E7" s="26" t="s">
         <v>77</v>
       </c>
-      <c r="F7" s="32" t="s">
+      <c r="F7" s="26" t="s">
         <v>78</v>
       </c>
-      <c r="G7" s="33" t="s">
+      <c r="G7" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="H7" s="19"/>
-      <c r="I7" s="32" t="s">
+      <c r="H7" s="13"/>
+      <c r="I7" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="8" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="25">
+      <c r="B8" s="19">
         <v>177</v>
       </c>
-      <c r="C8" s="18" t="s">
+      <c r="C8" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D8" s="28"/>
-      <c r="E8" s="32" t="s">
+      <c r="D8" s="22"/>
+      <c r="E8" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="F8" s="32" t="s">
+      <c r="F8" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="G8" s="33" t="s">
+      <c r="G8" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="H8" s="19"/>
-      <c r="I8" s="32" t="s">
+      <c r="H8" s="13"/>
+      <c r="I8" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="9" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="25">
+      <c r="B9" s="19">
         <v>178</v>
       </c>
-      <c r="C9" s="18" t="s">
+      <c r="C9" s="12" t="s">
         <v>83</v>
       </c>
-      <c r="D9" s="28"/>
-      <c r="E9" s="32" t="s">
+      <c r="D9" s="22"/>
+      <c r="E9" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="F9" s="32" t="s">
+      <c r="F9" s="26" t="s">
         <v>85</v>
       </c>
-      <c r="G9" s="33" t="s">
+      <c r="G9" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="H9" s="19"/>
-      <c r="I9" s="32" t="s">
+      <c r="H9" s="13"/>
+      <c r="I9" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="10" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B10" s="25">
+      <c r="B10" s="19">
         <v>179</v>
       </c>
-      <c r="C10" s="18" t="s">
+      <c r="C10" s="12" t="s">
         <v>86</v>
       </c>
-      <c r="D10" s="28"/>
-      <c r="E10" s="32" t="s">
+      <c r="D10" s="22"/>
+      <c r="E10" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="F10" s="32" t="s">
+      <c r="F10" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="G10" s="33" t="s">
+      <c r="G10" s="27" t="s">
         <v>79</v>
       </c>
-      <c r="H10" s="19"/>
-      <c r="I10" s="32" t="s">
+      <c r="H10" s="13"/>
+      <c r="I10" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B11" s="25">
+      <c r="B11" s="19">
         <v>180</v>
       </c>
-      <c r="C11" s="18" t="s">
+      <c r="C11" s="12" t="s">
         <v>89</v>
       </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="32" t="s">
+      <c r="D11" s="22"/>
+      <c r="E11" s="26" t="s">
         <v>90</v>
       </c>
-      <c r="F11" s="32" t="s">
+      <c r="F11" s="26" t="s">
         <v>91</v>
       </c>
-      <c r="G11" s="33" t="s">
+      <c r="G11" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="H11" s="19"/>
-      <c r="I11" s="32" t="s">
+      <c r="H11" s="13"/>
+      <c r="I11" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B12" s="25">
+      <c r="B12" s="19">
         <v>181</v>
       </c>
-      <c r="C12" s="18" t="s">
+      <c r="C12" s="12" t="s">
         <v>93</v>
       </c>
-      <c r="D12" s="28"/>
-      <c r="E12" s="32" t="s">
+      <c r="D12" s="22"/>
+      <c r="E12" s="26" t="s">
         <v>94</v>
       </c>
-      <c r="F12" s="32" t="s">
+      <c r="F12" s="26" t="s">
         <v>95</v>
       </c>
-      <c r="G12" s="33" t="s">
+      <c r="G12" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="H12" s="19"/>
-      <c r="I12" s="32" t="s">
+      <c r="H12" s="13"/>
+      <c r="I12" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="13" spans="2:9" ht="15.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B13" s="25">
+      <c r="B13" s="19">
         <v>183</v>
       </c>
-      <c r="C13" s="18" t="s">
+      <c r="C13" s="12" t="s">
         <v>96</v>
       </c>
-      <c r="D13" s="28"/>
-      <c r="E13" s="32" t="s">
+      <c r="D13" s="22"/>
+      <c r="E13" s="26" t="s">
         <v>97</v>
       </c>
-      <c r="F13" s="32" t="s">
+      <c r="F13" s="26" t="s">
         <v>98</v>
       </c>
-      <c r="G13" s="33" t="s">
+      <c r="G13" s="27" t="s">
         <v>92</v>
       </c>
-      <c r="H13" s="19"/>
-      <c r="I13" s="32" t="s">
+      <c r="H13" s="13"/>
+      <c r="I13" s="26" t="s">
         <v>65</v>
       </c>
     </row>
     <row r="14" spans="2:9" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B14" s="25">
+      <c r="B14" s="19">
         <v>459</v>
       </c>
-      <c r="C14" s="29" t="s">
+      <c r="C14" s="23" t="s">
         <v>99</v>
       </c>
-      <c r="D14" s="28"/>
-      <c r="E14" s="32" t="s">
+      <c r="D14" s="22"/>
+      <c r="E14" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="F14" s="32" t="s">
+      <c r="F14" s="26" t="s">
         <v>43</v>
       </c>
-      <c r="G14" s="33" t="s">
+      <c r="G14" s="27" t="s">
         <v>100</v>
       </c>
-      <c r="H14" s="19" t="s">
+      <c r="H14" s="13" t="s">
         <v>101</v>
       </c>
-      <c r="I14" s="32" t="s">
+      <c r="I14" s="26" t="s">
         <v>65</v>
       </c>
     </row>
@@ -1720,137 +2157,137 @@
       <c r="D17" s="2" t="s">
         <v>107</v>
       </c>
-      <c r="E17" s="20" t="s">
+      <c r="E17" s="14" t="s">
         <v>111</v>
       </c>
-      <c r="F17" s="20" t="s">
+      <c r="F17" s="14" t="s">
         <v>112</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="H17" s="23"/>
+      <c r="H17" s="17"/>
     </row>
     <row r="18" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B18" s="83" t="s">
+      <c r="B18" s="120" t="s">
         <v>6</v>
       </c>
-      <c r="C18" s="84"/>
-      <c r="D18" s="84"/>
-      <c r="E18" s="84"/>
-      <c r="F18" s="85"/>
-      <c r="G18" s="7" t="s">
+      <c r="C18" s="121"/>
+      <c r="D18" s="121"/>
+      <c r="E18" s="121"/>
+      <c r="F18" s="122"/>
+      <c r="G18" s="114" t="s">
         <v>102</v>
       </c>
-      <c r="H18" s="23"/>
+      <c r="H18" s="17"/>
     </row>
     <row r="19" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="15">
+      <c r="B19" s="9">
         <v>334</v>
       </c>
-      <c r="C19" s="26"/>
-      <c r="D19" s="16" t="s">
+      <c r="C19" s="20"/>
+      <c r="D19" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E19" s="17" t="s">
+      <c r="E19" s="11" t="s">
         <v>4</v>
       </c>
-      <c r="F19" s="17" t="s">
+      <c r="F19" s="11" t="s">
         <v>5</v>
       </c>
-      <c r="G19" s="8"/>
-      <c r="H19" s="23">
+      <c r="G19" s="115"/>
+      <c r="H19" s="17">
         <v>190</v>
       </c>
     </row>
     <row r="20" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B20" s="15">
+      <c r="B20" s="9">
         <v>335</v>
       </c>
-      <c r="C20" s="26"/>
-      <c r="D20" s="16" t="s">
+      <c r="C20" s="20"/>
+      <c r="D20" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="E20" s="17" t="s">
+      <c r="E20" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="F20" s="17" t="s">
+      <c r="F20" s="11" t="s">
         <v>9</v>
       </c>
-      <c r="G20" s="8"/>
-      <c r="H20" s="23"/>
+      <c r="G20" s="115"/>
+      <c r="H20" s="17"/>
     </row>
     <row r="21" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B21" s="15">
+      <c r="B21" s="9">
         <v>336</v>
       </c>
-      <c r="C21" s="26"/>
-      <c r="D21" s="16" t="s">
+      <c r="C21" s="20"/>
+      <c r="D21" s="10" t="s">
         <v>10</v>
       </c>
-      <c r="E21" s="17" t="s">
+      <c r="E21" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="F21" s="17" t="s">
+      <c r="F21" s="11" t="s">
         <v>12</v>
       </c>
-      <c r="G21" s="8"/>
-      <c r="H21" s="23"/>
+      <c r="G21" s="115"/>
+      <c r="H21" s="17"/>
     </row>
     <row r="22" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B22" s="15">
+      <c r="B22" s="9">
         <v>337</v>
       </c>
-      <c r="C22" s="26"/>
-      <c r="D22" s="16" t="s">
+      <c r="C22" s="20"/>
+      <c r="D22" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="E22" s="17" t="s">
+      <c r="E22" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="F22" s="17" t="s">
+      <c r="F22" s="11" t="s">
         <v>15</v>
       </c>
-      <c r="G22" s="8"/>
-      <c r="H22" s="23"/>
+      <c r="G22" s="115"/>
+      <c r="H22" s="17"/>
     </row>
     <row r="23" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B23" s="15">
+      <c r="B23" s="9">
         <v>458</v>
       </c>
-      <c r="C23" s="26" t="s">
+      <c r="C23" s="20" t="s">
         <v>109</v>
       </c>
-      <c r="D23" s="16" t="s">
+      <c r="D23" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="E23" s="17" t="s">
+      <c r="E23" s="11" t="s">
         <v>17</v>
       </c>
-      <c r="F23" s="17" t="s">
+      <c r="F23" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="G23" s="9"/>
-      <c r="H23" s="23"/>
+      <c r="G23" s="116"/>
+      <c r="H23" s="17"/>
     </row>
     <row r="24" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B24" s="83" t="s">
+      <c r="B24" s="120" t="s">
         <v>19</v>
       </c>
-      <c r="C24" s="84"/>
-      <c r="D24" s="84"/>
-      <c r="E24" s="84"/>
-      <c r="F24" s="85"/>
-      <c r="G24" s="10" t="s">
+      <c r="C24" s="121"/>
+      <c r="D24" s="121"/>
+      <c r="E24" s="121"/>
+      <c r="F24" s="122"/>
+      <c r="G24" s="117" t="s">
         <v>103</v>
       </c>
-      <c r="H24" s="23">
+      <c r="H24" s="17">
         <v>154</v>
       </c>
     </row>
     <row r="25" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B25" s="13"/>
-      <c r="C25" s="27"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="21"/>
       <c r="D25" s="3" t="s">
         <v>20</v>
       </c>
@@ -1860,12 +2297,12 @@
       <c r="F25" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="G25" s="11"/>
-      <c r="H25" s="23"/>
+      <c r="G25" s="118"/>
+      <c r="H25" s="17"/>
     </row>
     <row r="26" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B26" s="13"/>
-      <c r="C26" s="27"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="21"/>
       <c r="D26" s="3" t="s">
         <v>22</v>
       </c>
@@ -1875,12 +2312,12 @@
       <c r="F26" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="G26" s="11"/>
-      <c r="H26" s="23"/>
+      <c r="G26" s="118"/>
+      <c r="H26" s="17"/>
     </row>
     <row r="27" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B27" s="13"/>
-      <c r="C27" s="27"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="21"/>
       <c r="D27" s="3" t="s">
         <v>24</v>
       </c>
@@ -1890,12 +2327,12 @@
       <c r="F27" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="G27" s="11"/>
-      <c r="H27" s="23"/>
+      <c r="G27" s="118"/>
+      <c r="H27" s="17"/>
     </row>
     <row r="28" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B28" s="13"/>
-      <c r="C28" s="27"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="21"/>
       <c r="D28" s="3" t="s">
         <v>26</v>
       </c>
@@ -1905,66 +2342,66 @@
       <c r="F28" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="G28" s="12"/>
-      <c r="H28" s="23"/>
+      <c r="G28" s="119"/>
+      <c r="H28" s="17"/>
     </row>
     <row r="29" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B29" s="80" t="s">
+      <c r="B29" s="123" t="s">
         <v>105</v>
       </c>
-      <c r="C29" s="81"/>
-      <c r="D29" s="81"/>
-      <c r="E29" s="81"/>
-      <c r="F29" s="82"/>
-      <c r="G29" s="10" t="s">
+      <c r="C29" s="124"/>
+      <c r="D29" s="124"/>
+      <c r="E29" s="124"/>
+      <c r="F29" s="125"/>
+      <c r="G29" s="117" t="s">
         <v>104</v>
       </c>
-      <c r="H29" s="23">
+      <c r="H29" s="17">
         <v>128</v>
       </c>
     </row>
     <row r="30" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B30" s="13"/>
-      <c r="C30" s="48"/>
-      <c r="D30" s="49" t="s">
+      <c r="B30" s="7"/>
+      <c r="C30" s="42"/>
+      <c r="D30" s="43" t="s">
         <v>28</v>
       </c>
-      <c r="E30" s="50"/>
-      <c r="F30" s="49"/>
-      <c r="G30" s="11"/>
-      <c r="H30" s="23"/>
+      <c r="E30" s="44"/>
+      <c r="F30" s="43"/>
+      <c r="G30" s="118"/>
+      <c r="H30" s="17"/>
     </row>
     <row r="31" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="13"/>
-      <c r="C31" s="38"/>
-      <c r="D31" s="39" t="s">
+      <c r="B31" s="7"/>
+      <c r="C31" s="32"/>
+      <c r="D31" s="33" t="s">
         <v>29</v>
       </c>
-      <c r="E31" s="40"/>
-      <c r="F31" s="40" t="s">
+      <c r="E31" s="34"/>
+      <c r="F31" s="34" t="s">
         <v>30</v>
       </c>
-      <c r="G31" s="11"/>
-      <c r="H31" s="23"/>
+      <c r="G31" s="118"/>
+      <c r="H31" s="17"/>
     </row>
     <row r="32" spans="2:12" ht="30" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B32" s="13"/>
-      <c r="C32" s="41"/>
-      <c r="D32" s="42" t="s">
+      <c r="B32" s="7"/>
+      <c r="C32" s="35"/>
+      <c r="D32" s="36" t="s">
         <v>31</v>
       </c>
       <c r="E32" s="6"/>
       <c r="F32" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="G32" s="11"/>
-      <c r="H32" s="23" t="s">
+      <c r="G32" s="118"/>
+      <c r="H32" s="17" t="s">
         <v>113</v>
       </c>
       <c r="I32" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="J32" s="23" t="s">
+      <c r="J32" s="17" t="s">
         <v>122</v>
       </c>
       <c r="K32" s="5" t="s">
@@ -1975,29 +2412,29 @@
       </c>
     </row>
     <row r="33" spans="2:12" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B33" s="15">
+      <c r="B33" s="9">
         <v>82</v>
       </c>
-      <c r="C33" s="30" t="s">
+      <c r="C33" s="24" t="s">
         <v>74</v>
       </c>
-      <c r="D33" s="16" t="s">
+      <c r="D33" s="10" t="s">
         <v>33</v>
       </c>
-      <c r="E33" s="17" t="s">
+      <c r="E33" s="11" t="s">
         <v>34</v>
       </c>
-      <c r="F33" s="17" t="s">
+      <c r="F33" s="11" t="s">
         <v>35</v>
       </c>
-      <c r="G33" s="11"/>
-      <c r="H33" s="23" t="s">
+      <c r="G33" s="118"/>
+      <c r="H33" s="17" t="s">
         <v>118</v>
       </c>
       <c r="I33" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="J33" s="23" t="s">
+      <c r="J33" s="17" t="s">
         <v>120</v>
       </c>
       <c r="K33" s="5" t="s">
@@ -2008,29 +2445,29 @@
       </c>
     </row>
     <row r="34" spans="2:12" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B34" s="76">
+      <c r="B34" s="70">
         <v>67</v>
       </c>
-      <c r="C34" s="77" t="s">
+      <c r="C34" s="71" t="s">
         <v>66</v>
       </c>
-      <c r="D34" s="78" t="s">
+      <c r="D34" s="72" t="s">
         <v>36</v>
       </c>
-      <c r="E34" s="79" t="s">
+      <c r="E34" s="73" t="s">
         <v>37</v>
       </c>
-      <c r="F34" s="79" t="s">
+      <c r="F34" s="73" t="s">
         <v>38</v>
       </c>
-      <c r="G34" s="11"/>
-      <c r="H34" s="23" t="s">
+      <c r="G34" s="118"/>
+      <c r="H34" s="17" t="s">
         <v>124</v>
       </c>
       <c r="I34" s="5" t="s">
         <v>115</v>
       </c>
-      <c r="J34" s="23" t="s">
+      <c r="J34" s="17" t="s">
         <v>125</v>
       </c>
       <c r="K34" s="5" t="s">
@@ -2041,14 +2478,14 @@
       </c>
     </row>
     <row r="35" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B35" s="62"/>
-      <c r="C35" s="63"/>
-      <c r="D35" s="64" t="s">
+      <c r="B35" s="56"/>
+      <c r="C35" s="57"/>
+      <c r="D35" s="58" t="s">
         <v>39</v>
       </c>
-      <c r="E35" s="65"/>
-      <c r="F35" s="65"/>
-      <c r="G35" s="11"/>
+      <c r="E35" s="59"/>
+      <c r="F35" s="59"/>
+      <c r="G35" s="118"/>
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
@@ -2056,21 +2493,21 @@
       <c r="L35" s="5"/>
     </row>
     <row r="36" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B36" s="67">
+      <c r="B36" s="61">
         <v>28</v>
       </c>
-      <c r="C36" s="47" t="s">
+      <c r="C36" s="41" t="s">
         <v>61</v>
       </c>
-      <c r="D36" s="69" t="s">
+      <c r="D36" s="63" t="s">
         <v>40</v>
       </c>
-      <c r="E36" s="70"/>
-      <c r="F36" s="70" t="s">
+      <c r="E36" s="64"/>
+      <c r="F36" s="64" t="s">
         <v>41</v>
       </c>
-      <c r="G36" s="12"/>
-      <c r="H36" s="23" t="s">
+      <c r="G36" s="119"/>
+      <c r="H36" s="17" t="s">
         <v>114</v>
       </c>
       <c r="I36" s="5" t="s">
@@ -2087,40 +2524,40 @@
       </c>
     </row>
     <row r="37" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B37" s="80" t="s">
+      <c r="B37" s="123" t="s">
         <v>106</v>
       </c>
-      <c r="C37" s="81"/>
-      <c r="D37" s="81"/>
-      <c r="E37" s="81"/>
-      <c r="F37" s="82"/>
-      <c r="G37" s="10" t="s">
+      <c r="C37" s="124"/>
+      <c r="D37" s="124"/>
+      <c r="E37" s="124"/>
+      <c r="F37" s="125"/>
+      <c r="G37" s="117" t="s">
         <v>100</v>
       </c>
-      <c r="H37" s="23">
+      <c r="H37" s="17">
         <v>226</v>
       </c>
     </row>
     <row r="38" spans="2:12" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B38" s="67">
+      <c r="B38" s="61">
         <v>459</v>
       </c>
-      <c r="C38" s="68" t="s">
+      <c r="C38" s="62" t="s">
         <v>99</v>
       </c>
-      <c r="D38" s="69" t="s">
+      <c r="D38" s="63" t="s">
         <v>42</v>
       </c>
-      <c r="E38" s="70"/>
-      <c r="F38" s="70" t="s">
+      <c r="E38" s="64"/>
+      <c r="F38" s="64" t="s">
         <v>43</v>
       </c>
-      <c r="G38" s="11"/>
-      <c r="H38" s="23"/>
+      <c r="G38" s="118"/>
+      <c r="H38" s="17"/>
     </row>
     <row r="39" spans="2:12" ht="31.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="13"/>
-      <c r="C39" s="31" t="s">
+      <c r="B39" s="7"/>
+      <c r="C39" s="25" t="s">
         <v>110</v>
       </c>
       <c r="D39" s="3" t="s">
@@ -2130,36 +2567,36 @@
       <c r="F39" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="G39" s="11"/>
-      <c r="H39" s="23"/>
+      <c r="G39" s="118"/>
+      <c r="H39" s="17"/>
     </row>
     <row r="40" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B40" s="13"/>
-      <c r="C40" s="27"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="21"/>
       <c r="D40" s="3"/>
       <c r="E40" s="4"/>
       <c r="F40" s="4"/>
-      <c r="G40" s="12"/>
-      <c r="H40" s="23"/>
+      <c r="G40" s="119"/>
+      <c r="H40" s="17"/>
     </row>
     <row r="41" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B41" s="80" t="s">
+      <c r="B41" s="123" t="s">
         <v>58</v>
       </c>
-      <c r="C41" s="81"/>
-      <c r="D41" s="81"/>
-      <c r="E41" s="81"/>
-      <c r="F41" s="82"/>
-      <c r="G41" s="10" t="s">
+      <c r="C41" s="124"/>
+      <c r="D41" s="124"/>
+      <c r="E41" s="124"/>
+      <c r="F41" s="125"/>
+      <c r="G41" s="117" t="s">
         <v>73</v>
       </c>
-      <c r="H41" s="23">
+      <c r="H41" s="17">
         <v>383</v>
       </c>
     </row>
     <row r="42" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B42" s="13"/>
-      <c r="C42" s="27"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="21"/>
       <c r="D42" s="3" t="s">
         <v>46</v>
       </c>
@@ -2167,12 +2604,12 @@
       <c r="F42" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="G42" s="11"/>
-      <c r="H42" s="23"/>
+      <c r="G42" s="118"/>
+      <c r="H42" s="17"/>
     </row>
     <row r="43" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="13"/>
-      <c r="C43" s="27"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="21"/>
       <c r="D43" s="3" t="s">
         <v>48</v>
       </c>
@@ -2180,12 +2617,12 @@
       <c r="F43" s="4" t="s">
         <v>49</v>
       </c>
-      <c r="G43" s="11"/>
-      <c r="H43" s="23"/>
+      <c r="G43" s="118"/>
+      <c r="H43" s="17"/>
     </row>
     <row r="44" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B44" s="13"/>
-      <c r="C44" s="27"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="21"/>
       <c r="D44" s="3" t="s">
         <v>50</v>
       </c>
@@ -2193,14 +2630,14 @@
       <c r="F44" s="4" t="s">
         <v>51</v>
       </c>
-      <c r="G44" s="11"/>
-      <c r="H44" s="23"/>
+      <c r="G44" s="118"/>
+      <c r="H44" s="17"/>
     </row>
     <row r="45" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B45" s="13">
+      <c r="B45" s="7">
         <v>70</v>
       </c>
-      <c r="C45" s="27" t="s">
+      <c r="C45" s="21" t="s">
         <v>72</v>
       </c>
       <c r="D45" s="3" t="s">
@@ -2210,12 +2647,12 @@
       <c r="F45" s="4" t="s">
         <v>53</v>
       </c>
-      <c r="G45" s="11"/>
-      <c r="H45" s="23"/>
+      <c r="G45" s="118"/>
+      <c r="H45" s="17"/>
     </row>
     <row r="46" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B46" s="13"/>
-      <c r="C46" s="27"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="21"/>
       <c r="D46" s="3" t="s">
         <v>54</v>
       </c>
@@ -2223,12 +2660,12 @@
       <c r="F46" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="G46" s="11"/>
-      <c r="H46" s="23"/>
+      <c r="G46" s="118"/>
+      <c r="H46" s="17"/>
     </row>
     <row r="47" spans="2:12" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="13"/>
-      <c r="C47" s="27"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="21"/>
       <c r="D47" s="3" t="s">
         <v>56</v>
       </c>
@@ -2236,31 +2673,31 @@
       <c r="F47" s="4" t="s">
         <v>57</v>
       </c>
-      <c r="G47" s="12"/>
-      <c r="H47" s="23"/>
+      <c r="G47" s="119"/>
+      <c r="H47" s="17"/>
     </row>
     <row r="48" spans="2:12" x14ac:dyDescent="0.25">
       <c r="B48"/>
       <c r="C48"/>
-      <c r="H48" s="23"/>
+      <c r="H48" s="17"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>154</v>
       </c>
-      <c r="B49" s="14" t="s">
+      <c r="B49" s="8" t="s">
         <v>142</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>153</v>
       </c>
-      <c r="D49" s="56" t="s">
+      <c r="D49" s="50" t="s">
         <v>143</v>
       </c>
-      <c r="F49" s="57" t="s">
+      <c r="F49" s="51" t="s">
         <v>144</v>
       </c>
-      <c r="H49" s="23"/>
+      <c r="H49" s="17"/>
       <c r="I49" t="s">
         <v>145</v>
       </c>
@@ -2269,20 +2706,20 @@
       <c r="B50" s="5" t="s">
         <v>159</v>
       </c>
-      <c r="C50" s="59" t="s">
+      <c r="C50" s="53" t="s">
         <v>158</v>
       </c>
-      <c r="D50" s="34" t="s">
+      <c r="D50" s="28" t="s">
         <v>132</v>
       </c>
-      <c r="E50" s="35">
+      <c r="E50" s="29">
         <v>2002389</v>
       </c>
-      <c r="F50" s="36" t="s">
+      <c r="F50" s="30" t="s">
         <v>133</v>
       </c>
-      <c r="G50" s="37"/>
-      <c r="H50" s="23"/>
+      <c r="G50" s="31"/>
+      <c r="H50" s="17"/>
       <c r="I50" t="s">
         <v>157</v>
       </c>
@@ -2294,21 +2731,21 @@
       <c r="B51" s="5" t="s">
         <v>140</v>
       </c>
-      <c r="C51" s="58" t="s">
+      <c r="C51" s="52" t="s">
         <v>155</v>
       </c>
-      <c r="D51" s="43" t="s">
+      <c r="D51" s="37" t="s">
         <v>130</v>
       </c>
-      <c r="E51" s="44">
+      <c r="E51" s="38">
         <v>2013995</v>
       </c>
-      <c r="F51" s="45" t="s">
+      <c r="F51" s="39" t="s">
         <v>131</v>
       </c>
-      <c r="G51" s="46"/>
-      <c r="H51" s="46"/>
-      <c r="I51" s="66" t="s">
+      <c r="G51" s="40"/>
+      <c r="H51" s="40"/>
+      <c r="I51" s="60" t="s">
         <v>146</v>
       </c>
     </row>
@@ -2319,21 +2756,21 @@
       <c r="B52" s="5" t="s">
         <v>141</v>
       </c>
-      <c r="C52" s="51" t="s">
+      <c r="C52" s="45" t="s">
         <v>152</v>
       </c>
-      <c r="D52" s="52" t="s">
+      <c r="D52" s="46" t="s">
         <v>127</v>
       </c>
-      <c r="E52" s="53">
+      <c r="E52" s="47">
         <v>2059662</v>
       </c>
-      <c r="F52" s="54" t="s">
+      <c r="F52" s="48" t="s">
         <v>128</v>
       </c>
-      <c r="G52" s="55"/>
-      <c r="H52" s="55"/>
-      <c r="I52" s="66" t="s">
+      <c r="G52" s="49"/>
+      <c r="H52" s="49"/>
+      <c r="I52" s="60" t="s">
         <v>147</v>
       </c>
     </row>
@@ -2344,21 +2781,21 @@
       <c r="B53" s="5" t="s">
         <v>148</v>
       </c>
-      <c r="C53" s="71" t="s">
+      <c r="C53" s="65" t="s">
         <v>151</v>
       </c>
-      <c r="D53" s="72" t="s">
+      <c r="D53" s="66" t="s">
         <v>38</v>
       </c>
-      <c r="E53" s="73">
+      <c r="E53" s="67">
         <v>2114786</v>
       </c>
-      <c r="F53" s="74" t="s">
+      <c r="F53" s="68" t="s">
         <v>129</v>
       </c>
-      <c r="G53" s="75"/>
-      <c r="H53" s="75"/>
-      <c r="I53" s="66" t="s">
+      <c r="G53" s="69"/>
+      <c r="H53" s="69"/>
+      <c r="I53" s="60" t="s">
         <v>149</v>
       </c>
     </row>
@@ -2369,20 +2806,20 @@
       <c r="B54" s="5" t="s">
         <v>134</v>
       </c>
-      <c r="C54" s="60">
+      <c r="C54" s="54">
         <v>1040</v>
       </c>
-      <c r="D54" s="61" t="s">
+      <c r="D54" s="55" t="s">
         <v>136</v>
       </c>
-      <c r="E54" s="60">
+      <c r="E54" s="54">
         <v>2100031</v>
       </c>
-      <c r="F54" s="61" t="s">
+      <c r="F54" s="55" t="s">
         <v>138</v>
       </c>
-      <c r="G54" s="61"/>
-      <c r="I54" s="61" t="s">
+      <c r="G54" s="55"/>
+      <c r="I54" s="55" t="s">
         <v>136</v>
       </c>
     </row>
@@ -2405,7 +2842,7 @@
       <c r="F55" t="s">
         <v>139</v>
       </c>
-      <c r="I55" s="23" t="s">
+      <c r="I55" s="17" t="s">
         <v>137</v>
       </c>
     </row>
@@ -2428,27 +2865,1745 @@
       <c r="F56" t="s">
         <v>139</v>
       </c>
-      <c r="H56" s="23"/>
+      <c r="H56" s="17"/>
     </row>
     <row r="57" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="H57" s="23"/>
+      <c r="H57" s="17"/>
     </row>
     <row r="58" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="C58" s="23"/>
-      <c r="H58" s="23"/>
+      <c r="C58" s="17"/>
+      <c r="H58" s="17"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B24:F24"/>
+    <mergeCell ref="B29:F29"/>
+    <mergeCell ref="B37:F37"/>
+    <mergeCell ref="B41:F41"/>
     <mergeCell ref="G18:G23"/>
     <mergeCell ref="G24:G28"/>
     <mergeCell ref="G29:G36"/>
     <mergeCell ref="G37:G40"/>
     <mergeCell ref="G41:G47"/>
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B29:F29"/>
-    <mergeCell ref="B37:F37"/>
-    <mergeCell ref="B41:F41"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F654DB59-918E-4537-AC92-A13B048B16DE}">
+  <dimension ref="A2:J49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="68.5703125" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" style="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="74"/>
+    </row>
+    <row r="3" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="75" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3" s="76" t="s">
+        <v>161</v>
+      </c>
+      <c r="D3" s="76" t="s">
+        <v>162</v>
+      </c>
+      <c r="E3" s="76" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3" s="76" t="s">
+        <v>164</v>
+      </c>
+      <c r="G3" s="76" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="129" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="110" t="s">
+        <v>132</v>
+      </c>
+      <c r="F4" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="78">
+        <v>1421</v>
+      </c>
+      <c r="H4" s="112">
+        <f t="shared" ref="H4:H5" si="0">LEN(D4)</f>
+        <v>20</v>
+      </c>
+      <c r="I4" s="113" t="s">
+        <v>214</v>
+      </c>
+      <c r="J4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="130"/>
+      <c r="C5" s="77" t="s">
+        <v>167</v>
+      </c>
+      <c r="D5" s="79" t="s">
+        <v>218</v>
+      </c>
+      <c r="E5" s="110" t="s">
+        <v>130</v>
+      </c>
+      <c r="F5" s="78" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="78">
+        <v>1422</v>
+      </c>
+      <c r="H5" s="112">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="I5" s="113" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" s="130"/>
+      <c r="C6" s="105" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="106" t="s">
+        <v>216</v>
+      </c>
+      <c r="E6" s="111" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="108" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="108">
+        <v>82</v>
+      </c>
+      <c r="H6" s="112">
+        <f>LEN(D6)</f>
+        <v>41</v>
+      </c>
+      <c r="I6" s="113" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" s="130"/>
+      <c r="C7" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="106" t="s">
+        <v>219</v>
+      </c>
+      <c r="E7" s="111" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="108">
+        <v>67</v>
+      </c>
+      <c r="H7" s="112">
+        <f t="shared" ref="H7:H11" si="1">LEN(D7)</f>
+        <v>50</v>
+      </c>
+      <c r="I7" s="113" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="130"/>
+      <c r="C8" s="107" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="106" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="107" t="s">
+        <v>168</v>
+      </c>
+      <c r="F8" s="108" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="108">
+        <v>28</v>
+      </c>
+      <c r="H8" s="112">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="I8" s="113" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" s="130"/>
+      <c r="C9" s="77" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9" s="109" t="s">
+        <v>220</v>
+      </c>
+      <c r="E9" s="110" t="s">
+        <v>221</v>
+      </c>
+      <c r="F9" s="78" t="s">
+        <v>170</v>
+      </c>
+      <c r="G9" s="78">
+        <v>1299</v>
+      </c>
+      <c r="H9" s="112">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="I9" s="113"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" s="130"/>
+      <c r="C10" s="77" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E10" s="104">
+        <v>2063328</v>
+      </c>
+      <c r="F10" s="78" t="s">
+        <v>172</v>
+      </c>
+      <c r="G10" s="78">
+        <v>1246</v>
+      </c>
+      <c r="H10" s="112">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="I10" s="113" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" s="131"/>
+      <c r="C11" s="80" t="s">
+        <v>173</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" s="77" t="s">
+        <v>215</v>
+      </c>
+      <c r="F11" s="78" t="s">
+        <v>174</v>
+      </c>
+      <c r="G11" s="78">
+        <v>1040</v>
+      </c>
+      <c r="H11" s="112">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="I11" s="113" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="81"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="84"/>
+      <c r="F12" s="84"/>
+    </row>
+    <row r="13" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" s="132" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="85" t="s">
+        <v>175</v>
+      </c>
+      <c r="D13" s="86" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="86" t="s">
+        <v>176</v>
+      </c>
+      <c r="F13" s="87" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="87">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14" s="133"/>
+      <c r="C14" s="88" t="s">
+        <v>177</v>
+      </c>
+      <c r="D14" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="89" t="s">
+        <v>178</v>
+      </c>
+      <c r="F14" s="90" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="78"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="83"/>
+      <c r="C15" s="91"/>
+      <c r="D15" s="83"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16" s="132" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" s="86" t="s">
+        <v>179</v>
+      </c>
+      <c r="D16" s="86" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="86">
+        <v>6230361</v>
+      </c>
+      <c r="F16" s="92" t="s">
+        <v>180</v>
+      </c>
+      <c r="G16" s="87"/>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17" s="134"/>
+      <c r="C17" s="89" t="s">
+        <v>181</v>
+      </c>
+      <c r="D17" s="89" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="89">
+        <v>6250340</v>
+      </c>
+      <c r="F17" s="93" t="s">
+        <v>182</v>
+      </c>
+      <c r="G17" s="78"/>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" s="134"/>
+      <c r="C18" s="89" t="s">
+        <v>183</v>
+      </c>
+      <c r="D18" s="89" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="89">
+        <v>6240369</v>
+      </c>
+      <c r="F18" s="93" t="s">
+        <v>184</v>
+      </c>
+      <c r="G18" s="78"/>
+    </row>
+    <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1</v>
+      </c>
+      <c r="B19" s="133"/>
+      <c r="C19" s="89" t="s">
+        <v>185</v>
+      </c>
+      <c r="D19" s="89" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="89">
+        <v>6260359</v>
+      </c>
+      <c r="F19" s="93" t="s">
+        <v>186</v>
+      </c>
+      <c r="G19" s="78"/>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="83"/>
+      <c r="C20" s="91"/>
+      <c r="D20" s="83"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="83"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1</v>
+      </c>
+      <c r="B21" s="129" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" s="94" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21" s="86" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="95" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="95">
+        <v>334</v>
+      </c>
+      <c r="H21" s="112"/>
+      <c r="I21" s="113"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22" s="130"/>
+      <c r="C22" s="77" t="s">
+        <v>188</v>
+      </c>
+      <c r="D22" s="89" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="78" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="78">
+        <v>335</v>
+      </c>
+      <c r="H22" s="112"/>
+      <c r="I22" s="113"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" s="130"/>
+      <c r="C23" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="D23" s="89" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="77" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="78" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="78">
+        <v>336</v>
+      </c>
+      <c r="H23" s="112"/>
+      <c r="I23" s="113"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>1</v>
+      </c>
+      <c r="B24" s="130"/>
+      <c r="C24" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="D24" s="89" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="78" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="78">
+        <v>337</v>
+      </c>
+      <c r="H24" s="112"/>
+      <c r="I24" s="113"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>1</v>
+      </c>
+      <c r="B25" s="131"/>
+      <c r="C25" s="77" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="89" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="78" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="78">
+        <v>458</v>
+      </c>
+      <c r="H25" s="112"/>
+      <c r="I25" s="113"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="83"/>
+      <c r="C26" s="91"/>
+      <c r="D26" s="83"/>
+      <c r="E26" s="83"/>
+      <c r="F26" s="83"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" s="132" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="86" t="s">
+        <v>191</v>
+      </c>
+      <c r="D27" s="86" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="86"/>
+      <c r="F27" s="92" t="s">
+        <v>192</v>
+      </c>
+      <c r="G27" s="87"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" s="134"/>
+      <c r="C28" s="89" t="s">
+        <v>193</v>
+      </c>
+      <c r="D28" s="89" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="89"/>
+      <c r="F28" s="93" t="s">
+        <v>194</v>
+      </c>
+      <c r="G28" s="78"/>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>1</v>
+      </c>
+      <c r="B29" s="134"/>
+      <c r="C29" s="89" t="s">
+        <v>195</v>
+      </c>
+      <c r="D29" s="89" t="s">
+        <v>50</v>
+      </c>
+      <c r="E29" s="89"/>
+      <c r="F29" s="93" t="s">
+        <v>196</v>
+      </c>
+      <c r="G29" s="78"/>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>1</v>
+      </c>
+      <c r="B30" s="134"/>
+      <c r="C30" s="89" t="s">
+        <v>197</v>
+      </c>
+      <c r="D30" s="89" t="s">
+        <v>52</v>
+      </c>
+      <c r="E30" s="89"/>
+      <c r="F30" s="93" t="s">
+        <v>198</v>
+      </c>
+      <c r="G30" s="78"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>1</v>
+      </c>
+      <c r="B31" s="134"/>
+      <c r="C31" s="89" t="s">
+        <v>199</v>
+      </c>
+      <c r="D31" s="89" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31" s="89"/>
+      <c r="F31" s="97" t="s">
+        <v>200</v>
+      </c>
+      <c r="G31" s="78"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>1</v>
+      </c>
+      <c r="B32" s="135"/>
+      <c r="C32" s="89" t="s">
+        <v>201</v>
+      </c>
+      <c r="D32" s="89" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" s="89"/>
+      <c r="F32" s="93" t="s">
+        <v>202</v>
+      </c>
+      <c r="G32" s="78"/>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="98"/>
+      <c r="C33" s="90"/>
+      <c r="D33" s="89"/>
+      <c r="E33" s="89"/>
+      <c r="F33" s="89"/>
+      <c r="G33" s="78"/>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" s="99" t="s">
+        <v>203</v>
+      </c>
+      <c r="C34" s="77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D34" s="3"/>
+      <c r="E34" s="77" t="s">
+        <v>69</v>
+      </c>
+      <c r="F34" s="100" t="s">
+        <v>204</v>
+      </c>
+      <c r="G34" s="78"/>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="83"/>
+      <c r="C35" s="91"/>
+      <c r="D35" s="83"/>
+      <c r="E35" s="83"/>
+      <c r="F35" s="83"/>
+      <c r="G35" s="78"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>1</v>
+      </c>
+      <c r="B36" s="126" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="94" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" s="96"/>
+      <c r="E36" s="94" t="s">
+        <v>77</v>
+      </c>
+      <c r="F36" s="101" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="78"/>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37" s="127"/>
+      <c r="C37" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="3"/>
+      <c r="E37" s="77" t="s">
+        <v>81</v>
+      </c>
+      <c r="F37" s="100" t="s">
+        <v>206</v>
+      </c>
+      <c r="G37" s="78"/>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" s="127"/>
+      <c r="C38" s="77" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="3"/>
+      <c r="E38" s="77" t="s">
+        <v>84</v>
+      </c>
+      <c r="F38" s="100" t="s">
+        <v>207</v>
+      </c>
+      <c r="G38" s="78"/>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" s="128"/>
+      <c r="C39" s="77" t="s">
+        <v>86</v>
+      </c>
+      <c r="D39" s="3"/>
+      <c r="E39" s="77" t="s">
+        <v>87</v>
+      </c>
+      <c r="F39" s="100" t="s">
+        <v>208</v>
+      </c>
+      <c r="G39" s="78"/>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="83"/>
+      <c r="C40" s="91"/>
+      <c r="D40" s="83"/>
+      <c r="E40" s="83"/>
+      <c r="F40" s="83"/>
+      <c r="G40" s="102"/>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>1</v>
+      </c>
+      <c r="B41" s="126" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="94" t="s">
+        <v>89</v>
+      </c>
+      <c r="D41" s="96"/>
+      <c r="E41" s="94" t="s">
+        <v>90</v>
+      </c>
+      <c r="F41" s="101" t="s">
+        <v>209</v>
+      </c>
+      <c r="G41" s="103"/>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>1</v>
+      </c>
+      <c r="B42" s="127"/>
+      <c r="C42" s="77" t="s">
+        <v>93</v>
+      </c>
+      <c r="D42" s="3"/>
+      <c r="E42" s="77" t="s">
+        <v>94</v>
+      </c>
+      <c r="F42" s="100" t="s">
+        <v>210</v>
+      </c>
+      <c r="G42" s="78"/>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>1</v>
+      </c>
+      <c r="B43" s="128"/>
+      <c r="C43" s="77" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" s="3"/>
+      <c r="E43" s="77" t="s">
+        <v>97</v>
+      </c>
+      <c r="F43" s="100" t="s">
+        <v>211</v>
+      </c>
+      <c r="G43" s="78"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <f>SUM(A4:A43)</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <f>13*100</f>
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <f>+A48/33</f>
+        <v>39.393939393939391</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B4:B11"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="B36:B39"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DDFFEA8D-C314-4915-82E5-443D53F193C8}">
+  <dimension ref="A2:J49"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="15.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="71.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="68.5703125" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.42578125" style="5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.85546875" style="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="74"/>
+    </row>
+    <row r="3" spans="1:10" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="75" t="s">
+        <v>160</v>
+      </c>
+      <c r="C3" s="76" t="s">
+        <v>161</v>
+      </c>
+      <c r="D3" s="76" t="s">
+        <v>162</v>
+      </c>
+      <c r="E3" s="76" t="s">
+        <v>163</v>
+      </c>
+      <c r="F3" s="76" t="s">
+        <v>164</v>
+      </c>
+      <c r="G3" s="76" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>1</v>
+      </c>
+      <c r="B4" s="129" t="s">
+        <v>165</v>
+      </c>
+      <c r="C4" s="77" t="s">
+        <v>166</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E4" s="110" t="s">
+        <v>132</v>
+      </c>
+      <c r="F4" s="78" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="78">
+        <v>1421</v>
+      </c>
+      <c r="H4" s="137">
+        <f t="shared" ref="H4:H5" si="0">LEN(D4)</f>
+        <v>20</v>
+      </c>
+      <c r="I4" s="137" t="s">
+        <v>214</v>
+      </c>
+      <c r="J4" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>1</v>
+      </c>
+      <c r="B5" s="130"/>
+      <c r="C5" s="77" t="s">
+        <v>167</v>
+      </c>
+      <c r="D5" s="79" t="s">
+        <v>218</v>
+      </c>
+      <c r="E5" s="110" t="s">
+        <v>130</v>
+      </c>
+      <c r="F5" s="78" t="s">
+        <v>32</v>
+      </c>
+      <c r="G5" s="78">
+        <v>1422</v>
+      </c>
+      <c r="H5" s="137">
+        <f t="shared" si="0"/>
+        <v>50</v>
+      </c>
+      <c r="I5" s="137" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>1</v>
+      </c>
+      <c r="B6" s="130"/>
+      <c r="C6" s="105" t="s">
+        <v>74</v>
+      </c>
+      <c r="D6" s="106" t="s">
+        <v>216</v>
+      </c>
+      <c r="E6" s="111" t="s">
+        <v>127</v>
+      </c>
+      <c r="F6" s="108" t="s">
+        <v>35</v>
+      </c>
+      <c r="G6" s="108">
+        <v>82</v>
+      </c>
+      <c r="H6" s="137">
+        <f>LEN(D6)</f>
+        <v>41</v>
+      </c>
+      <c r="I6" s="137" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>1</v>
+      </c>
+      <c r="B7" s="130"/>
+      <c r="C7" s="36" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" s="106" t="s">
+        <v>219</v>
+      </c>
+      <c r="E7" s="111" t="s">
+        <v>38</v>
+      </c>
+      <c r="F7" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="G7" s="108">
+        <v>67</v>
+      </c>
+      <c r="H7" s="137">
+        <f t="shared" ref="H7:H11" si="1">LEN(D7)</f>
+        <v>50</v>
+      </c>
+      <c r="I7" s="137" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>1</v>
+      </c>
+      <c r="B8" s="130"/>
+      <c r="C8" s="107" t="s">
+        <v>61</v>
+      </c>
+      <c r="D8" s="106" t="s">
+        <v>40</v>
+      </c>
+      <c r="E8" s="107" t="s">
+        <v>168</v>
+      </c>
+      <c r="F8" s="108" t="s">
+        <v>41</v>
+      </c>
+      <c r="G8" s="108">
+        <v>28</v>
+      </c>
+      <c r="H8" s="137">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="I8" s="137" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>1</v>
+      </c>
+      <c r="B9" s="130"/>
+      <c r="C9" s="77" t="s">
+        <v>169</v>
+      </c>
+      <c r="D9" s="109" t="s">
+        <v>220</v>
+      </c>
+      <c r="E9" s="110" t="s">
+        <v>221</v>
+      </c>
+      <c r="F9" s="78" t="s">
+        <v>170</v>
+      </c>
+      <c r="G9" s="78">
+        <v>1299</v>
+      </c>
+      <c r="H9" s="137">
+        <f t="shared" si="1"/>
+        <v>50</v>
+      </c>
+      <c r="I9" s="137"/>
+    </row>
+    <row r="10" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>1</v>
+      </c>
+      <c r="B10" s="130"/>
+      <c r="C10" s="77" t="s">
+        <v>171</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E10" s="104">
+        <v>2063328</v>
+      </c>
+      <c r="F10" s="78" t="s">
+        <v>172</v>
+      </c>
+      <c r="G10" s="78">
+        <v>1246</v>
+      </c>
+      <c r="H10" s="137">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="I10" s="137" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>1</v>
+      </c>
+      <c r="B11" s="131"/>
+      <c r="C11" s="80" t="s">
+        <v>173</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E11" s="77" t="s">
+        <v>215</v>
+      </c>
+      <c r="F11" s="78" t="s">
+        <v>174</v>
+      </c>
+      <c r="G11" s="78">
+        <v>1040</v>
+      </c>
+      <c r="H11" s="137">
+        <f t="shared" si="1"/>
+        <v>16</v>
+      </c>
+      <c r="I11" s="137" t="s">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="81"/>
+      <c r="C12" s="82"/>
+      <c r="D12" s="83"/>
+      <c r="E12" s="84"/>
+      <c r="F12" s="84"/>
+    </row>
+    <row r="13" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>1</v>
+      </c>
+      <c r="B13" s="132" t="s">
+        <v>100</v>
+      </c>
+      <c r="C13" s="85" t="s">
+        <v>175</v>
+      </c>
+      <c r="D13" s="86" t="s">
+        <v>42</v>
+      </c>
+      <c r="E13" s="86" t="s">
+        <v>176</v>
+      </c>
+      <c r="F13" s="87" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="87">
+        <v>459</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>1</v>
+      </c>
+      <c r="B14" s="133"/>
+      <c r="C14" s="88" t="s">
+        <v>177</v>
+      </c>
+      <c r="D14" s="89" t="s">
+        <v>44</v>
+      </c>
+      <c r="E14" s="89" t="s">
+        <v>178</v>
+      </c>
+      <c r="F14" s="90" t="s">
+        <v>45</v>
+      </c>
+      <c r="G14" s="78"/>
+    </row>
+    <row r="15" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B15" s="83"/>
+      <c r="C15" s="91"/>
+      <c r="D15" s="83"/>
+      <c r="E15" s="83"/>
+      <c r="F15" s="83"/>
+    </row>
+    <row r="16" spans="1:10" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>1</v>
+      </c>
+      <c r="B16" s="132" t="s">
+        <v>103</v>
+      </c>
+      <c r="C16" s="136" t="s">
+        <v>226</v>
+      </c>
+      <c r="D16" s="86" t="s">
+        <v>20</v>
+      </c>
+      <c r="E16" s="136" t="s">
+        <v>222</v>
+      </c>
+      <c r="F16" s="92" t="s">
+        <v>180</v>
+      </c>
+      <c r="G16" s="87">
+        <v>1453</v>
+      </c>
+      <c r="H16" s="137">
+        <v>7.2300000000000003E-2</v>
+      </c>
+      <c r="I16" s="137" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>1</v>
+      </c>
+      <c r="B17" s="134"/>
+      <c r="C17" s="109" t="s">
+        <v>228</v>
+      </c>
+      <c r="D17" s="89" t="s">
+        <v>22</v>
+      </c>
+      <c r="E17" s="109" t="s">
+        <v>223</v>
+      </c>
+      <c r="F17" s="93" t="s">
+        <v>182</v>
+      </c>
+      <c r="G17" s="78">
+        <v>1454</v>
+      </c>
+      <c r="H17" s="137">
+        <v>9.2299999999999993E-2</v>
+      </c>
+      <c r="I17" s="137" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>1</v>
+      </c>
+      <c r="B18" s="134"/>
+      <c r="C18" s="109" t="s">
+        <v>227</v>
+      </c>
+      <c r="D18" s="89" t="s">
+        <v>24</v>
+      </c>
+      <c r="E18" s="109" t="s">
+        <v>224</v>
+      </c>
+      <c r="F18" s="93" t="s">
+        <v>184</v>
+      </c>
+      <c r="G18" s="78">
+        <v>1459</v>
+      </c>
+      <c r="H18" s="137">
+        <v>8.3089999999999997E-2</v>
+      </c>
+      <c r="I18" s="137" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>1</v>
+      </c>
+      <c r="B19" s="133"/>
+      <c r="C19" s="109" t="s">
+        <v>229</v>
+      </c>
+      <c r="D19" s="89" t="s">
+        <v>26</v>
+      </c>
+      <c r="E19" s="109" t="s">
+        <v>225</v>
+      </c>
+      <c r="F19" s="93" t="s">
+        <v>186</v>
+      </c>
+      <c r="G19" s="78">
+        <v>1460</v>
+      </c>
+      <c r="H19" s="137">
+        <v>8.8870000000000005E-2</v>
+      </c>
+      <c r="I19" s="137" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B20" s="83"/>
+      <c r="C20" s="91"/>
+      <c r="D20" s="83"/>
+      <c r="E20" s="83"/>
+      <c r="F20" s="83"/>
+    </row>
+    <row r="21" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>1</v>
+      </c>
+      <c r="B21" s="129" t="s">
+        <v>102</v>
+      </c>
+      <c r="C21" s="94" t="s">
+        <v>187</v>
+      </c>
+      <c r="D21" s="86" t="s">
+        <v>3</v>
+      </c>
+      <c r="E21" s="94" t="s">
+        <v>4</v>
+      </c>
+      <c r="F21" s="95" t="s">
+        <v>5</v>
+      </c>
+      <c r="G21" s="95">
+        <v>334</v>
+      </c>
+      <c r="H21" s="137"/>
+      <c r="I21" s="137"/>
+    </row>
+    <row r="22" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>1</v>
+      </c>
+      <c r="B22" s="130"/>
+      <c r="C22" s="77" t="s">
+        <v>188</v>
+      </c>
+      <c r="D22" s="89" t="s">
+        <v>7</v>
+      </c>
+      <c r="E22" s="77" t="s">
+        <v>8</v>
+      </c>
+      <c r="F22" s="78" t="s">
+        <v>9</v>
+      </c>
+      <c r="G22" s="78">
+        <v>335</v>
+      </c>
+      <c r="H22" s="137"/>
+      <c r="I22" s="137"/>
+    </row>
+    <row r="23" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>1</v>
+      </c>
+      <c r="B23" s="130"/>
+      <c r="C23" s="77" t="s">
+        <v>189</v>
+      </c>
+      <c r="D23" s="89" t="s">
+        <v>10</v>
+      </c>
+      <c r="E23" s="77" t="s">
+        <v>11</v>
+      </c>
+      <c r="F23" s="78" t="s">
+        <v>12</v>
+      </c>
+      <c r="G23" s="78">
+        <v>336</v>
+      </c>
+      <c r="H23" s="137"/>
+      <c r="I23" s="137"/>
+    </row>
+    <row r="24" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>1</v>
+      </c>
+      <c r="B24" s="130"/>
+      <c r="C24" s="77" t="s">
+        <v>190</v>
+      </c>
+      <c r="D24" s="89" t="s">
+        <v>13</v>
+      </c>
+      <c r="E24" s="77" t="s">
+        <v>14</v>
+      </c>
+      <c r="F24" s="78" t="s">
+        <v>15</v>
+      </c>
+      <c r="G24" s="78">
+        <v>337</v>
+      </c>
+      <c r="H24" s="137"/>
+      <c r="I24" s="137"/>
+    </row>
+    <row r="25" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>1</v>
+      </c>
+      <c r="B25" s="131"/>
+      <c r="C25" s="77" t="s">
+        <v>109</v>
+      </c>
+      <c r="D25" s="89" t="s">
+        <v>16</v>
+      </c>
+      <c r="E25" s="77" t="s">
+        <v>17</v>
+      </c>
+      <c r="F25" s="78" t="s">
+        <v>18</v>
+      </c>
+      <c r="G25" s="78">
+        <v>458</v>
+      </c>
+      <c r="H25" s="137"/>
+      <c r="I25" s="137"/>
+    </row>
+    <row r="26" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B26" s="83"/>
+      <c r="C26" s="91"/>
+      <c r="D26" s="83"/>
+      <c r="E26" s="83"/>
+      <c r="F26" s="83"/>
+    </row>
+    <row r="27" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>1</v>
+      </c>
+      <c r="B27" s="132" t="s">
+        <v>73</v>
+      </c>
+      <c r="C27" s="86" t="s">
+        <v>191</v>
+      </c>
+      <c r="D27" s="86" t="s">
+        <v>46</v>
+      </c>
+      <c r="E27" s="86"/>
+      <c r="F27" s="92" t="s">
+        <v>192</v>
+      </c>
+      <c r="G27" s="87"/>
+    </row>
+    <row r="28" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>1</v>
+      </c>
+      <c r="B28" s="134"/>
+      <c r="C28" s="89" t="s">
+        <v>193</v>
+      </c>
+      <c r="D28" s="89" t="s">
+        <v>48</v>
+      </c>
+      <c r="E28" s="89"/>
+      <c r="F28" s="93" t="s">
+        <v>194</v>
+      </c>
+      <c r="G28" s="78"/>
+      <c r="H28">
+        <v>16.420000000000002</v>
+      </c>
+      <c r="I28" s="17" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A29">
+        <v>1</v>
+      </c>
+      <c r="B29" s="134"/>
+      <c r="C29" s="89" t="s">
+        <v>195</v>
+      </c>
+      <c r="D29" s="89" t="s">
+        <v>50</v>
+      </c>
+      <c r="E29" s="89"/>
+      <c r="F29" s="93" t="s">
+        <v>196</v>
+      </c>
+      <c r="G29" s="78"/>
+      <c r="H29">
+        <v>16.420000000000002</v>
+      </c>
+      <c r="I29" s="17" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A30">
+        <v>1</v>
+      </c>
+      <c r="B30" s="134"/>
+      <c r="C30" s="89" t="s">
+        <v>197</v>
+      </c>
+      <c r="D30" s="89" t="s">
+        <v>52</v>
+      </c>
+      <c r="E30" s="89"/>
+      <c r="F30" s="93" t="s">
+        <v>198</v>
+      </c>
+      <c r="G30" s="78"/>
+    </row>
+    <row r="31" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A31">
+        <v>1</v>
+      </c>
+      <c r="B31" s="134"/>
+      <c r="C31" s="89" t="s">
+        <v>199</v>
+      </c>
+      <c r="D31" s="89" t="s">
+        <v>54</v>
+      </c>
+      <c r="E31" s="89"/>
+      <c r="F31" s="97" t="s">
+        <v>200</v>
+      </c>
+      <c r="G31" s="78"/>
+    </row>
+    <row r="32" spans="1:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A32">
+        <v>1</v>
+      </c>
+      <c r="B32" s="135"/>
+      <c r="C32" s="89" t="s">
+        <v>201</v>
+      </c>
+      <c r="D32" s="89" t="s">
+        <v>56</v>
+      </c>
+      <c r="E32" s="89"/>
+      <c r="F32" s="93" t="s">
+        <v>202</v>
+      </c>
+      <c r="G32" s="78"/>
+    </row>
+    <row r="33" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B33" s="98"/>
+      <c r="C33" s="90"/>
+      <c r="D33" s="89"/>
+      <c r="E33" s="89"/>
+      <c r="F33" s="89"/>
+      <c r="G33" s="78"/>
+    </row>
+    <row r="34" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A34">
+        <v>1</v>
+      </c>
+      <c r="B34" s="99" t="s">
+        <v>203</v>
+      </c>
+      <c r="C34" s="77" t="s">
+        <v>68</v>
+      </c>
+      <c r="D34" s="3"/>
+      <c r="E34" s="77" t="s">
+        <v>69</v>
+      </c>
+      <c r="F34" s="100" t="s">
+        <v>204</v>
+      </c>
+      <c r="G34" s="78"/>
+    </row>
+    <row r="35" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B35" s="83"/>
+      <c r="C35" s="91"/>
+      <c r="D35" s="83"/>
+      <c r="E35" s="83"/>
+      <c r="F35" s="83"/>
+      <c r="G35" s="78"/>
+    </row>
+    <row r="36" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A36">
+        <v>1</v>
+      </c>
+      <c r="B36" s="126" t="s">
+        <v>79</v>
+      </c>
+      <c r="C36" s="94" t="s">
+        <v>76</v>
+      </c>
+      <c r="D36" s="96"/>
+      <c r="E36" s="94" t="s">
+        <v>77</v>
+      </c>
+      <c r="F36" s="101" t="s">
+        <v>205</v>
+      </c>
+      <c r="G36" s="78"/>
+    </row>
+    <row r="37" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A37">
+        <v>1</v>
+      </c>
+      <c r="B37" s="127"/>
+      <c r="C37" s="77" t="s">
+        <v>80</v>
+      </c>
+      <c r="D37" s="3"/>
+      <c r="E37" s="77" t="s">
+        <v>81</v>
+      </c>
+      <c r="F37" s="100" t="s">
+        <v>206</v>
+      </c>
+      <c r="G37" s="78"/>
+    </row>
+    <row r="38" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A38">
+        <v>1</v>
+      </c>
+      <c r="B38" s="127"/>
+      <c r="C38" s="77" t="s">
+        <v>83</v>
+      </c>
+      <c r="D38" s="3"/>
+      <c r="E38" s="77" t="s">
+        <v>84</v>
+      </c>
+      <c r="F38" s="100" t="s">
+        <v>207</v>
+      </c>
+      <c r="G38" s="78"/>
+    </row>
+    <row r="39" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A39">
+        <v>1</v>
+      </c>
+      <c r="B39" s="128"/>
+      <c r="C39" s="77" t="s">
+        <v>86</v>
+      </c>
+      <c r="D39" s="3"/>
+      <c r="E39" s="77" t="s">
+        <v>87</v>
+      </c>
+      <c r="F39" s="100" t="s">
+        <v>208</v>
+      </c>
+      <c r="G39" s="78"/>
+    </row>
+    <row r="40" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B40" s="83"/>
+      <c r="C40" s="91"/>
+      <c r="D40" s="83"/>
+      <c r="E40" s="83"/>
+      <c r="F40" s="83"/>
+      <c r="G40" s="102"/>
+    </row>
+    <row r="41" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A41">
+        <v>1</v>
+      </c>
+      <c r="B41" s="126" t="s">
+        <v>92</v>
+      </c>
+      <c r="C41" s="94" t="s">
+        <v>89</v>
+      </c>
+      <c r="D41" s="96"/>
+      <c r="E41" s="94" t="s">
+        <v>90</v>
+      </c>
+      <c r="F41" s="101" t="s">
+        <v>209</v>
+      </c>
+      <c r="G41" s="103"/>
+    </row>
+    <row r="42" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A42">
+        <v>1</v>
+      </c>
+      <c r="B42" s="127"/>
+      <c r="C42" s="77" t="s">
+        <v>93</v>
+      </c>
+      <c r="D42" s="3"/>
+      <c r="E42" s="77" t="s">
+        <v>94</v>
+      </c>
+      <c r="F42" s="100" t="s">
+        <v>210</v>
+      </c>
+      <c r="G42" s="78"/>
+    </row>
+    <row r="43" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A43">
+        <v>1</v>
+      </c>
+      <c r="B43" s="128"/>
+      <c r="C43" s="77" t="s">
+        <v>96</v>
+      </c>
+      <c r="D43" s="3"/>
+      <c r="E43" s="77" t="s">
+        <v>97</v>
+      </c>
+      <c r="F43" s="100" t="s">
+        <v>211</v>
+      </c>
+      <c r="G43" s="78"/>
+    </row>
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A45">
+        <f>SUM(A4:A43)</f>
+        <v>33</v>
+      </c>
+    </row>
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A46">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A48">
+        <f>13*100</f>
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49">
+        <f>+A48/33</f>
+        <v>39.393939393939391</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="7">
+    <mergeCell ref="B41:B43"/>
+    <mergeCell ref="B4:B11"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="B16:B19"/>
+    <mergeCell ref="B21:B25"/>
+    <mergeCell ref="B27:B32"/>
+    <mergeCell ref="B36:B39"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>